<commit_message>
fix orphography in rpd.xlsx
</commit_message>
<xml_diff>
--- a/data/RPD.xlsx
+++ b/data/RPD.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\June\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\June\Курсы повышения квалификации\ИТМО\repos\ITMO_AI_Top_Teaching\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0139DDC-5439-42A4-9D49-5440237F6E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E44C704-13E9-430B-BD51-D91C274C5165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Главный раздел РПД" sheetId="1" r:id="rId1"/>
@@ -909,9 +909,6 @@
     <t>Б; С</t>
   </si>
   <si>
-    <t>Модуль1. Выборка, разведочный и непараметрический анализ данных</t>
-  </si>
-  <si>
     <t>Занятие 1.1. Выборка, эмпирическое распределение и описательная статистика</t>
   </si>
   <si>
@@ -1087,6 +1084,9 @@
   </si>
   <si>
     <t>Строит непараметрические и параметрические модели для низкоразмерных распределений (двухмерных, трехмерных).</t>
+  </si>
+  <si>
+    <t>Модуль 1. Выборка, разведочный и непараметрический анализ данных</t>
   </si>
 </sst>
 </file>
@@ -1464,7 +1464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1705,6 +1705,33 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1731,30 +1758,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1782,6 +1785,99 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1791,9 +1887,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1806,102 +1899,39 @@
     <xf numFmtId="0" fontId="15" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1910,39 +1940,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2129,35 +2126,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="17" hidden="1" customHeight="1">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="98" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
+      <c r="B1" s="98"/>
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="98"/>
+      <c r="H1" s="98"/>
       <c r="I1" s="45"/>
       <c r="J1" s="45"/>
       <c r="K1" s="16"/>
-      <c r="L1" s="89" t="s">
+      <c r="L1" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="89"/>
+      <c r="M1" s="98"/>
     </row>
     <row r="2" spans="1:13" ht="15" hidden="1" customHeight="1">
-      <c r="A2" s="98" t="s">
+      <c r="A2" s="99" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="98"/>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
+      <c r="B2" s="99"/>
+      <c r="C2" s="99"/>
+      <c r="D2" s="99"/>
+      <c r="E2" s="99"/>
+      <c r="F2" s="99"/>
+      <c r="G2" s="99"/>
+      <c r="H2" s="99"/>
       <c r="I2" s="46"/>
       <c r="J2" s="46"/>
       <c r="K2" s="16"/>
@@ -2170,16 +2167,16 @@
       </c>
     </row>
     <row r="3" spans="1:13" ht="29" hidden="1" customHeight="1">
-      <c r="A3" s="99" t="s">
+      <c r="A3" s="100" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="99"/>
-      <c r="C3" s="99"/>
-      <c r="D3" s="99"/>
-      <c r="E3" s="99"/>
-      <c r="F3" s="99"/>
-      <c r="G3" s="99"/>
-      <c r="H3" s="99"/>
+      <c r="B3" s="100"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="100"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="100"/>
+      <c r="G3" s="100"/>
+      <c r="H3" s="100"/>
       <c r="I3" s="47"/>
       <c r="J3" s="47"/>
       <c r="K3" s="16"/>
@@ -2192,16 +2189,16 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="15" hidden="1" customHeight="1">
-      <c r="A4" s="100" t="s">
+      <c r="A4" s="101" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="100"/>
-      <c r="C4" s="100"/>
-      <c r="D4" s="100"/>
-      <c r="E4" s="100"/>
-      <c r="F4" s="100"/>
-      <c r="G4" s="100"/>
-      <c r="H4" s="100"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="101"/>
+      <c r="D4" s="101"/>
+      <c r="E4" s="101"/>
+      <c r="F4" s="101"/>
+      <c r="G4" s="101"/>
+      <c r="H4" s="101"/>
       <c r="I4" s="48"/>
       <c r="J4" s="48"/>
       <c r="K4" s="16"/>
@@ -2233,16 +2230,16 @@
         <v>13</v>
       </c>
       <c r="G5" s="22" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H5" s="23" t="s">
         <v>14</v>
       </c>
       <c r="I5" s="49" t="s">
+        <v>317</v>
+      </c>
+      <c r="J5" s="49" t="s">
         <v>318</v>
-      </c>
-      <c r="J5" s="49" t="s">
-        <v>319</v>
       </c>
       <c r="K5" s="16"/>
       <c r="L5" s="19" t="s">
@@ -2254,7 +2251,7 @@
     </row>
     <row r="6" spans="1:13" ht="30.4" customHeight="1">
       <c r="A6" s="55" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="B6" s="24" t="s">
         <v>16</v>
@@ -2270,17 +2267,17 @@
         <v>17</v>
       </c>
       <c r="F6" s="71" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G6" s="71"/>
       <c r="H6" s="72" t="s">
         <v>288</v>
       </c>
       <c r="I6" s="73" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="J6" s="73" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="K6" s="16"/>
       <c r="L6" s="16"/>
@@ -2291,7 +2288,7 @@
     </row>
     <row r="7" spans="1:13" ht="57" customHeight="1">
       <c r="A7" s="54" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B7" s="56" t="s">
         <v>268</v>
@@ -2302,23 +2299,23 @@
       <c r="D7" s="59">
         <v>2</v>
       </c>
-      <c r="E7" s="92" t="s">
+      <c r="E7" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="92" t="s">
+      <c r="F7" s="81" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="94" t="s">
+      <c r="G7" s="84" t="s">
         <v>229</v>
       </c>
       <c r="H7" s="61" t="s">
         <v>21</v>
       </c>
       <c r="I7" s="61" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J7" s="61" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K7" s="16"/>
       <c r="L7" s="16"/>
@@ -2326,7 +2323,7 @@
     </row>
     <row r="8" spans="1:13" ht="40.5" customHeight="1">
       <c r="A8" s="54" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B8" s="57" t="s">
         <v>269</v>
@@ -2337,28 +2334,28 @@
       <c r="D8" s="61">
         <v>2</v>
       </c>
-      <c r="E8" s="159"/>
-      <c r="F8" s="159"/>
-      <c r="G8" s="160"/>
+      <c r="E8" s="82"/>
+      <c r="F8" s="82"/>
+      <c r="G8" s="85"/>
       <c r="H8" s="61" t="s">
         <v>21</v>
       </c>
       <c r="I8" s="61" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J8" s="61" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K8" s="16"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
     </row>
     <row r="9" spans="1:13" ht="17" customHeight="1">
-      <c r="A9" s="103" t="s">
-        <v>292</v>
-      </c>
-      <c r="B9" s="105" t="s">
-        <v>330</v>
+      <c r="A9" s="104" t="s">
+        <v>291</v>
+      </c>
+      <c r="B9" s="106" t="s">
+        <v>329</v>
       </c>
       <c r="C9" s="59" t="s">
         <v>20</v>
@@ -2366,44 +2363,44 @@
       <c r="D9" s="59">
         <v>2</v>
       </c>
-      <c r="E9" s="159"/>
-      <c r="F9" s="159"/>
-      <c r="G9" s="160"/>
-      <c r="H9" s="92" t="s">
+      <c r="E9" s="82"/>
+      <c r="F9" s="82"/>
+      <c r="G9" s="85"/>
+      <c r="H9" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="92" t="s">
-        <v>331</v>
-      </c>
-      <c r="J9" s="92" t="s">
-        <v>333</v>
+      <c r="I9" s="81" t="s">
+        <v>330</v>
+      </c>
+      <c r="J9" s="81" t="s">
+        <v>332</v>
       </c>
       <c r="K9" s="16"/>
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
     </row>
     <row r="10" spans="1:13" ht="39" customHeight="1">
-      <c r="A10" s="104"/>
-      <c r="B10" s="106"/>
+      <c r="A10" s="105"/>
+      <c r="B10" s="107"/>
       <c r="C10" s="59" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="59">
         <v>2</v>
       </c>
-      <c r="E10" s="93"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="95"/>
-      <c r="H10" s="93"/>
-      <c r="I10" s="93"/>
-      <c r="J10" s="93"/>
+      <c r="E10" s="83"/>
+      <c r="F10" s="83"/>
+      <c r="G10" s="86"/>
+      <c r="H10" s="83"/>
+      <c r="I10" s="83"/>
+      <c r="J10" s="83"/>
       <c r="K10" s="16"/>
       <c r="L10" s="16"/>
       <c r="M10" s="16"/>
     </row>
     <row r="11" spans="1:13" ht="58.5" customHeight="1">
       <c r="A11" s="54" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B11" s="57" t="s">
         <v>270</v>
@@ -2421,16 +2418,16 @@
         <v>27</v>
       </c>
       <c r="G11" s="75" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="H11" s="61" t="s">
         <v>19</v>
       </c>
       <c r="I11" s="61" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J11" s="61" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K11" s="16"/>
       <c r="L11" s="16"/>
@@ -2438,7 +2435,7 @@
     </row>
     <row r="12" spans="1:13" ht="32.25" customHeight="1">
       <c r="A12" s="55" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B12" s="58" t="s">
         <v>16</v>
@@ -2461,10 +2458,10 @@
         <v>288</v>
       </c>
       <c r="I12" s="50" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="J12" s="50" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="K12" s="16"/>
       <c r="L12" s="16"/>
@@ -2472,7 +2469,7 @@
     </row>
     <row r="13" spans="1:13" ht="32" customHeight="1">
       <c r="A13" s="54" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B13" s="57" t="s">
         <v>271</v>
@@ -2483,23 +2480,23 @@
       <c r="D13" s="61">
         <v>2</v>
       </c>
-      <c r="E13" s="92" t="s">
+      <c r="E13" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="92" t="s">
+      <c r="F13" s="81" t="s">
         <v>18</v>
       </c>
-      <c r="G13" s="81" t="s">
+      <c r="G13" s="89" t="s">
         <v>229</v>
       </c>
       <c r="H13" s="61" t="s">
         <v>21</v>
       </c>
       <c r="I13" s="70" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J13" s="63" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K13" s="16"/>
       <c r="L13" s="16"/>
@@ -2507,7 +2504,7 @@
     </row>
     <row r="14" spans="1:13" ht="34" customHeight="1">
       <c r="A14" s="54" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B14" s="56" t="s">
         <v>272</v>
@@ -2518,17 +2515,17 @@
       <c r="D14" s="59">
         <v>2</v>
       </c>
-      <c r="E14" s="96"/>
-      <c r="F14" s="96"/>
-      <c r="G14" s="97"/>
+      <c r="E14" s="82"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="90"/>
       <c r="H14" s="59" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="59" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J14" s="60" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K14" s="16"/>
       <c r="L14" s="16"/>
@@ -2536,7 +2533,7 @@
     </row>
     <row r="15" spans="1:13" ht="34" customHeight="1">
       <c r="A15" s="54" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B15" s="57" t="s">
         <v>273</v>
@@ -2547,17 +2544,17 @@
       <c r="D15" s="61">
         <v>2</v>
       </c>
-      <c r="E15" s="96"/>
-      <c r="F15" s="96"/>
-      <c r="G15" s="97"/>
+      <c r="E15" s="82"/>
+      <c r="F15" s="82"/>
+      <c r="G15" s="90"/>
       <c r="H15" s="61" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="76" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J15" s="77" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K15" s="16"/>
       <c r="L15" s="16"/>
@@ -2565,7 +2562,7 @@
     </row>
     <row r="16" spans="1:13" ht="68.5" customHeight="1">
       <c r="A16" s="54" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B16" s="56" t="s">
         <v>274</v>
@@ -2576,17 +2573,17 @@
       <c r="D16" s="59">
         <v>2</v>
       </c>
-      <c r="E16" s="93"/>
-      <c r="F16" s="93"/>
-      <c r="G16" s="82"/>
+      <c r="E16" s="83"/>
+      <c r="F16" s="83"/>
+      <c r="G16" s="91"/>
       <c r="H16" s="59" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="59" t="s">
+        <v>330</v>
+      </c>
+      <c r="J16" s="60" t="s">
         <v>331</v>
-      </c>
-      <c r="J16" s="60" t="s">
-        <v>332</v>
       </c>
       <c r="K16" s="16"/>
       <c r="L16" s="16"/>
@@ -2594,7 +2591,7 @@
     </row>
     <row r="17" spans="1:13" ht="33.9" customHeight="1">
       <c r="A17" s="55" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B17" s="58" t="s">
         <v>16</v>
@@ -2617,10 +2614,10 @@
         <v>288</v>
       </c>
       <c r="I17" s="50" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="J17" s="50" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="K17" s="16"/>
       <c r="L17" s="16"/>
@@ -2628,7 +2625,7 @@
     </row>
     <row r="18" spans="1:13" ht="34" customHeight="1">
       <c r="A18" s="54" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B18" s="57" t="s">
         <v>275</v>
@@ -2639,23 +2636,23 @@
       <c r="D18" s="61">
         <v>4</v>
       </c>
-      <c r="E18" s="92" t="s">
+      <c r="E18" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="F18" s="92" t="s">
+      <c r="F18" s="81" t="s">
         <v>27</v>
       </c>
-      <c r="G18" s="81" t="s">
+      <c r="G18" s="89" t="s">
         <v>234</v>
       </c>
       <c r="H18" s="61" t="s">
         <v>21</v>
       </c>
       <c r="I18" s="76" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J18" s="77" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K18" s="16"/>
       <c r="L18" s="16"/>
@@ -2663,10 +2660,10 @@
     </row>
     <row r="19" spans="1:13" ht="34" customHeight="1">
       <c r="A19" s="54" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B19" s="56" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C19" s="59" t="s">
         <v>22</v>
@@ -2674,17 +2671,17 @@
       <c r="D19" s="59">
         <v>6</v>
       </c>
-      <c r="E19" s="93"/>
-      <c r="F19" s="93"/>
-      <c r="G19" s="82"/>
+      <c r="E19" s="83"/>
+      <c r="F19" s="83"/>
+      <c r="G19" s="91"/>
       <c r="H19" s="59" t="s">
         <v>19</v>
       </c>
       <c r="I19" s="59" t="s">
+        <v>330</v>
+      </c>
+      <c r="J19" s="60" t="s">
         <v>331</v>
-      </c>
-      <c r="J19" s="60" t="s">
-        <v>332</v>
       </c>
       <c r="K19" s="16"/>
       <c r="L19" s="16"/>
@@ -2692,7 +2689,7 @@
     </row>
     <row r="20" spans="1:13" ht="114.5" customHeight="1">
       <c r="A20" s="54" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B20" s="57" t="s">
         <v>276</v>
@@ -2710,16 +2707,16 @@
         <v>28</v>
       </c>
       <c r="G20" s="74" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H20" s="61" t="s">
         <v>19</v>
       </c>
       <c r="I20" s="76" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J20" s="77" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K20" s="16"/>
       <c r="L20" s="16"/>
@@ -2727,7 +2724,7 @@
     </row>
     <row r="21" spans="1:13" ht="30" customHeight="1">
       <c r="A21" s="55" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B21" s="58" t="s">
         <v>16</v>
@@ -2747,13 +2744,13 @@
       </c>
       <c r="G21" s="25"/>
       <c r="H21" s="26" t="s">
-        <v>31</v>
+        <v>283</v>
       </c>
       <c r="I21" s="50" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="J21" s="50" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="K21" s="16"/>
       <c r="L21" s="16"/>
@@ -2761,7 +2758,7 @@
     </row>
     <row r="22" spans="1:13" ht="47" customHeight="1">
       <c r="A22" s="54" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B22" s="57" t="s">
         <v>277</v>
@@ -2772,23 +2769,23 @@
       <c r="D22" s="61">
         <v>2</v>
       </c>
-      <c r="E22" s="92" t="s">
+      <c r="E22" s="81" t="s">
         <v>29</v>
       </c>
-      <c r="F22" s="92" t="s">
+      <c r="F22" s="81" t="s">
         <v>32</v>
       </c>
-      <c r="G22" s="81" t="s">
+      <c r="G22" s="89" t="s">
         <v>239</v>
       </c>
       <c r="H22" s="61" t="s">
         <v>21</v>
       </c>
       <c r="I22" s="76" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J22" s="77" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K22" s="16"/>
       <c r="L22" s="16"/>
@@ -2796,7 +2793,7 @@
     </row>
     <row r="23" spans="1:13" ht="35" customHeight="1">
       <c r="A23" s="54" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B23" s="56" t="s">
         <v>278</v>
@@ -2807,17 +2804,17 @@
       <c r="D23" s="59">
         <v>2</v>
       </c>
-      <c r="E23" s="93"/>
-      <c r="F23" s="93"/>
-      <c r="G23" s="82"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="83"/>
+      <c r="G23" s="91"/>
       <c r="H23" s="59" t="s">
         <v>19</v>
       </c>
       <c r="I23" s="59" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J23" s="60" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K23" s="16"/>
       <c r="L23" s="16"/>
@@ -2825,7 +2822,7 @@
     </row>
     <row r="24" spans="1:13" ht="55.5" customHeight="1">
       <c r="A24" s="54" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B24" s="57" t="s">
         <v>279</v>
@@ -2836,23 +2833,23 @@
       <c r="D24" s="61">
         <v>4</v>
       </c>
-      <c r="E24" s="92" t="s">
+      <c r="E24" s="81" t="s">
         <v>29</v>
       </c>
-      <c r="F24" s="92" t="s">
+      <c r="F24" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="G24" s="81" t="s">
+      <c r="G24" s="89" t="s">
         <v>243</v>
       </c>
       <c r="H24" s="61" t="s">
         <v>21</v>
       </c>
       <c r="I24" s="76" t="s">
+        <v>330</v>
+      </c>
+      <c r="J24" s="77" t="s">
         <v>331</v>
-      </c>
-      <c r="J24" s="77" t="s">
-        <v>332</v>
       </c>
       <c r="K24" s="16"/>
       <c r="L24" s="16"/>
@@ -2860,7 +2857,7 @@
     </row>
     <row r="25" spans="1:13" ht="33" customHeight="1">
       <c r="A25" s="54" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B25" s="56" t="s">
         <v>280</v>
@@ -2871,17 +2868,17 @@
       <c r="D25" s="59">
         <v>2</v>
       </c>
-      <c r="E25" s="93"/>
-      <c r="F25" s="93"/>
-      <c r="G25" s="82"/>
+      <c r="E25" s="83"/>
+      <c r="F25" s="83"/>
+      <c r="G25" s="91"/>
       <c r="H25" s="59" t="s">
         <v>21</v>
       </c>
       <c r="I25" s="59" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J25" s="59" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K25" s="16"/>
       <c r="L25" s="16"/>
@@ -2889,7 +2886,7 @@
     </row>
     <row r="26" spans="1:13" ht="32.65" customHeight="1">
       <c r="A26" s="55" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B26" s="58" t="s">
         <v>16</v>
@@ -2912,10 +2909,10 @@
         <v>283</v>
       </c>
       <c r="I26" s="50" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="J26" s="50" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="K26" s="16"/>
       <c r="L26" s="16"/>
@@ -2923,7 +2920,7 @@
     </row>
     <row r="27" spans="1:13" ht="68.5" customHeight="1">
       <c r="A27" s="54" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B27" s="56" t="s">
         <v>281</v>
@@ -2947,10 +2944,10 @@
         <v>21</v>
       </c>
       <c r="I27" s="59" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J27" s="77" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K27" s="16"/>
       <c r="L27" s="16"/>
@@ -2958,10 +2955,10 @@
     </row>
     <row r="28" spans="1:13" ht="113.5" customHeight="1">
       <c r="A28" s="54" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B28" s="56" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C28" s="59" t="s">
         <v>22</v>
@@ -2982,10 +2979,10 @@
         <v>21</v>
       </c>
       <c r="I28" s="59" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J28" s="77" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K28" s="16"/>
       <c r="L28" s="16"/>
@@ -2993,7 +2990,7 @@
     </row>
     <row r="29" spans="1:13" ht="115.5" customHeight="1">
       <c r="A29" s="54" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B29" s="57" t="s">
         <v>287</v>
@@ -3017,10 +3014,10 @@
         <v>19</v>
       </c>
       <c r="I29" s="76" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J29" s="76" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K29" s="16"/>
       <c r="L29" s="16"/>
@@ -3028,7 +3025,7 @@
     </row>
     <row r="30" spans="1:13" ht="29.25" customHeight="1">
       <c r="A30" s="55" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B30" s="58" t="s">
         <v>16</v>
@@ -3048,10 +3045,10 @@
       </c>
       <c r="G30" s="25"/>
       <c r="H30" s="26" t="s">
-        <v>19</v>
+        <v>283</v>
       </c>
       <c r="I30" s="50" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="J30" s="50"/>
       <c r="K30" s="16"/>
@@ -3060,7 +3057,7 @@
     </row>
     <row r="31" spans="1:13" ht="63" customHeight="1">
       <c r="A31" s="54" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B31" s="56" t="s">
         <v>284</v>
@@ -3071,23 +3068,23 @@
       <c r="D31" s="59">
         <v>4</v>
       </c>
-      <c r="E31" s="83" t="s">
+      <c r="E31" s="92" t="s">
         <v>24</v>
       </c>
-      <c r="F31" s="83" t="s">
+      <c r="F31" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="G31" s="86" t="s">
+      <c r="G31" s="95" t="s">
         <v>257</v>
       </c>
       <c r="H31" s="59" t="s">
         <v>21</v>
       </c>
       <c r="I31" s="59" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J31" s="60" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K31" s="16"/>
       <c r="L31" s="16"/>
@@ -3095,7 +3092,7 @@
     </row>
     <row r="32" spans="1:13" ht="44.5" customHeight="1">
       <c r="A32" s="54" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B32" s="57" t="s">
         <v>285</v>
@@ -3106,27 +3103,27 @@
       <c r="D32" s="61">
         <v>4</v>
       </c>
-      <c r="E32" s="84"/>
-      <c r="F32" s="84"/>
-      <c r="G32" s="87"/>
+      <c r="E32" s="93"/>
+      <c r="F32" s="93"/>
+      <c r="G32" s="96"/>
       <c r="H32" s="61" t="s">
         <v>19</v>
       </c>
       <c r="I32" s="61" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J32" s="62" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K32" s="16"/>
       <c r="L32" s="16"/>
       <c r="M32" s="16"/>
     </row>
     <row r="33" spans="1:13" ht="29.5" customHeight="1">
-      <c r="A33" s="101" t="s">
-        <v>314</v>
-      </c>
-      <c r="B33" s="90" t="s">
+      <c r="A33" s="102" t="s">
+        <v>313</v>
+      </c>
+      <c r="B33" s="87" t="s">
         <v>286</v>
       </c>
       <c r="C33" s="59" t="s">
@@ -3135,42 +3132,42 @@
       <c r="D33" s="59">
         <v>4</v>
       </c>
-      <c r="E33" s="84"/>
-      <c r="F33" s="84"/>
-      <c r="G33" s="87"/>
+      <c r="E33" s="93"/>
+      <c r="F33" s="93"/>
+      <c r="G33" s="96"/>
       <c r="H33" s="59" t="s">
         <v>21</v>
       </c>
       <c r="I33" s="59" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J33" s="60" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K33" s="16"/>
       <c r="L33" s="16"/>
       <c r="M33" s="16"/>
     </row>
     <row r="34" spans="1:13" ht="29.5" customHeight="1">
-      <c r="A34" s="102"/>
-      <c r="B34" s="91"/>
+      <c r="A34" s="103"/>
+      <c r="B34" s="88"/>
       <c r="C34" s="59" t="s">
         <v>22</v>
       </c>
       <c r="D34" s="59">
         <v>2</v>
       </c>
-      <c r="E34" s="84"/>
-      <c r="F34" s="84"/>
-      <c r="G34" s="87"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="93"/>
+      <c r="G34" s="96"/>
       <c r="H34" s="61" t="s">
         <v>21</v>
       </c>
       <c r="I34" s="61" t="s">
+        <v>330</v>
+      </c>
+      <c r="J34" s="61" t="s">
         <v>331</v>
-      </c>
-      <c r="J34" s="61" t="s">
-        <v>332</v>
       </c>
       <c r="K34" s="16"/>
       <c r="L34" s="16"/>
@@ -3178,7 +3175,7 @@
     </row>
     <row r="35" spans="1:13" ht="43.15" customHeight="1">
       <c r="A35" s="54" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B35" s="57" t="s">
         <v>35</v>
@@ -3189,17 +3186,17 @@
       <c r="D35" s="61">
         <v>2</v>
       </c>
-      <c r="E35" s="85"/>
-      <c r="F35" s="85"/>
-      <c r="G35" s="88"/>
+      <c r="E35" s="94"/>
+      <c r="F35" s="94"/>
+      <c r="G35" s="97"/>
       <c r="H35" s="59" t="s">
         <v>19</v>
       </c>
       <c r="I35" s="59" t="s">
+        <v>330</v>
+      </c>
+      <c r="J35" s="60" t="s">
         <v>331</v>
-      </c>
-      <c r="J35" s="60" t="s">
-        <v>332</v>
       </c>
       <c r="K35" s="16"/>
       <c r="L35" s="16"/>
@@ -3227,10 +3224,10 @@
       <c r="G36" s="29"/>
       <c r="H36" s="30"/>
       <c r="I36" s="30" t="s">
+        <v>343</v>
+      </c>
+      <c r="J36" s="51" t="s">
         <v>344</v>
-      </c>
-      <c r="J36" s="51" t="s">
-        <v>345</v>
       </c>
       <c r="K36" s="16"/>
       <c r="L36" s="16"/>
@@ -3304,11 +3301,14 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="E7:E10"/>
-    <mergeCell ref="F7:F10"/>
-    <mergeCell ref="G7:G10"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
     <mergeCell ref="J9:J10"/>
     <mergeCell ref="E13:E16"/>
     <mergeCell ref="F13:F16"/>
@@ -3316,24 +3316,21 @@
     <mergeCell ref="E18:E19"/>
     <mergeCell ref="F18:F19"/>
     <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="E7:E10"/>
+    <mergeCell ref="F7:F10"/>
+    <mergeCell ref="G7:G10"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="I9:I10"/>
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="F22:F23"/>
     <mergeCell ref="G22:G23"/>
     <mergeCell ref="E24:E25"/>
     <mergeCell ref="F24:F25"/>
-    <mergeCell ref="H9:H10"/>
     <mergeCell ref="G24:G25"/>
     <mergeCell ref="E31:E35"/>
     <mergeCell ref="F31:F35"/>
     <mergeCell ref="G31:G35"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3352,226 +3349,226 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17" customHeight="1">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="139" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
     </row>
     <row r="2" spans="1:8" ht="16" customHeight="1">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="140" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="108"/>
-      <c r="C2" s="108"/>
-      <c r="D2" s="108"/>
-      <c r="E2" s="108"/>
-      <c r="F2" s="108"/>
-      <c r="G2" s="108"/>
-      <c r="H2" s="108"/>
+      <c r="B2" s="140"/>
+      <c r="C2" s="140"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="140"/>
+      <c r="F2" s="140"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="109" t="s">
+      <c r="A4" s="141" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="110"/>
-      <c r="C4" s="109" t="s">
+      <c r="B4" s="123"/>
+      <c r="C4" s="141" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="110"/>
-      <c r="E4" s="109" t="s">
+      <c r="D4" s="123"/>
+      <c r="E4" s="141" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="110"/>
-      <c r="G4" s="109" t="s">
+      <c r="F4" s="123"/>
+      <c r="G4" s="141" t="s">
         <v>50</v>
       </c>
-      <c r="H4" s="110"/>
+      <c r="H4" s="123"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="111" t="s">
+      <c r="A5" s="142" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="112"/>
-      <c r="C5" s="111" t="s">
+      <c r="B5" s="143"/>
+      <c r="C5" s="142" t="s">
         <v>52</v>
       </c>
-      <c r="D5" s="112"/>
-      <c r="E5" s="111" t="s">
+      <c r="D5" s="143"/>
+      <c r="E5" s="142" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="112"/>
-      <c r="G5" s="111" t="s">
+      <c r="F5" s="143"/>
+      <c r="G5" s="142" t="s">
         <v>54</v>
       </c>
-      <c r="H5" s="112"/>
+      <c r="H5" s="143"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="113"/>
-      <c r="B6" s="114"/>
-      <c r="C6" s="113"/>
-      <c r="D6" s="114"/>
-      <c r="E6" s="113"/>
-      <c r="F6" s="114"/>
-      <c r="G6" s="113"/>
-      <c r="H6" s="114"/>
+      <c r="A6" s="144"/>
+      <c r="B6" s="145"/>
+      <c r="C6" s="144"/>
+      <c r="D6" s="145"/>
+      <c r="E6" s="144"/>
+      <c r="F6" s="145"/>
+      <c r="G6" s="144"/>
+      <c r="H6" s="145"/>
     </row>
     <row r="8" spans="1:8" ht="15.5">
-      <c r="A8" s="115" t="s">
+      <c r="A8" s="117" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="115"/>
-      <c r="C8" s="115"/>
-      <c r="D8" s="115"/>
-      <c r="E8" s="115"/>
-      <c r="F8" s="115"/>
-      <c r="G8" s="115"/>
-      <c r="H8" s="115"/>
+      <c r="B8" s="117"/>
+      <c r="C8" s="117"/>
+      <c r="D8" s="117"/>
+      <c r="E8" s="117"/>
+      <c r="F8" s="117"/>
+      <c r="G8" s="117"/>
+      <c r="H8" s="117"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="116" t="s">
+      <c r="A9" s="130" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="117"/>
-      <c r="C9" s="117"/>
-      <c r="D9" s="117"/>
-      <c r="E9" s="117"/>
-      <c r="F9" s="117"/>
-      <c r="G9" s="117"/>
-      <c r="H9" s="118"/>
+      <c r="B9" s="131"/>
+      <c r="C9" s="131"/>
+      <c r="D9" s="131"/>
+      <c r="E9" s="131"/>
+      <c r="F9" s="131"/>
+      <c r="G9" s="131"/>
+      <c r="H9" s="132"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="119"/>
-      <c r="B10" s="120"/>
-      <c r="C10" s="120"/>
-      <c r="D10" s="120"/>
-      <c r="E10" s="120"/>
-      <c r="F10" s="120"/>
-      <c r="G10" s="120"/>
-      <c r="H10" s="121"/>
+      <c r="A10" s="133"/>
+      <c r="B10" s="134"/>
+      <c r="C10" s="134"/>
+      <c r="D10" s="134"/>
+      <c r="E10" s="134"/>
+      <c r="F10" s="134"/>
+      <c r="G10" s="134"/>
+      <c r="H10" s="135"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="122"/>
-      <c r="B11" s="123"/>
-      <c r="C11" s="123"/>
-      <c r="D11" s="123"/>
-      <c r="E11" s="123"/>
-      <c r="F11" s="123"/>
-      <c r="G11" s="123"/>
-      <c r="H11" s="124"/>
+      <c r="A11" s="136"/>
+      <c r="B11" s="137"/>
+      <c r="C11" s="137"/>
+      <c r="D11" s="137"/>
+      <c r="E11" s="137"/>
+      <c r="F11" s="137"/>
+      <c r="G11" s="137"/>
+      <c r="H11" s="138"/>
     </row>
     <row r="13" spans="1:8" ht="15.5">
-      <c r="A13" s="115" t="s">
+      <c r="A13" s="117" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="115"/>
-      <c r="C13" s="115"/>
-      <c r="D13" s="115"/>
-      <c r="E13" s="115"/>
-      <c r="F13" s="115"/>
-      <c r="G13" s="115"/>
-      <c r="H13" s="115"/>
+      <c r="B13" s="117"/>
+      <c r="C13" s="117"/>
+      <c r="D13" s="117"/>
+      <c r="E13" s="117"/>
+      <c r="F13" s="117"/>
+      <c r="G13" s="117"/>
+      <c r="H13" s="117"/>
     </row>
     <row r="14" spans="1:8" ht="17" customHeight="1">
       <c r="A14" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="125" t="s">
+      <c r="B14" s="124" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="126"/>
-      <c r="D14" s="126"/>
-      <c r="E14" s="126"/>
-      <c r="F14" s="126"/>
-      <c r="G14" s="126"/>
-      <c r="H14" s="127"/>
+      <c r="C14" s="125"/>
+      <c r="D14" s="125"/>
+      <c r="E14" s="125"/>
+      <c r="F14" s="125"/>
+      <c r="G14" s="125"/>
+      <c r="H14" s="126"/>
     </row>
     <row r="15" spans="1:8" ht="17" customHeight="1">
       <c r="A15" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="128" t="s">
+      <c r="B15" s="127" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="129"/>
-      <c r="D15" s="129"/>
-      <c r="E15" s="129"/>
-      <c r="F15" s="129"/>
-      <c r="G15" s="129"/>
-      <c r="H15" s="130"/>
+      <c r="C15" s="128"/>
+      <c r="D15" s="128"/>
+      <c r="E15" s="128"/>
+      <c r="F15" s="128"/>
+      <c r="G15" s="128"/>
+      <c r="H15" s="129"/>
     </row>
     <row r="16" spans="1:8" ht="17" customHeight="1">
       <c r="A16" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="125" t="s">
+      <c r="B16" s="124" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="126"/>
-      <c r="D16" s="126"/>
-      <c r="E16" s="126"/>
-      <c r="F16" s="126"/>
-      <c r="G16" s="126"/>
-      <c r="H16" s="127"/>
+      <c r="C16" s="125"/>
+      <c r="D16" s="125"/>
+      <c r="E16" s="125"/>
+      <c r="F16" s="125"/>
+      <c r="G16" s="125"/>
+      <c r="H16" s="126"/>
     </row>
     <row r="17" spans="1:8" ht="17" customHeight="1">
       <c r="A17" s="39" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="128" t="s">
+      <c r="B17" s="127" t="s">
         <v>64</v>
       </c>
-      <c r="C17" s="129"/>
-      <c r="D17" s="129"/>
-      <c r="E17" s="129"/>
-      <c r="F17" s="129"/>
-      <c r="G17" s="129"/>
-      <c r="H17" s="130"/>
+      <c r="C17" s="128"/>
+      <c r="D17" s="128"/>
+      <c r="E17" s="128"/>
+      <c r="F17" s="128"/>
+      <c r="G17" s="128"/>
+      <c r="H17" s="129"/>
     </row>
     <row r="18" spans="1:8" ht="17" customHeight="1">
       <c r="A18" s="39" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="125" t="s">
+      <c r="B18" s="124" t="s">
         <v>66</v>
       </c>
-      <c r="C18" s="126"/>
-      <c r="D18" s="126"/>
-      <c r="E18" s="126"/>
-      <c r="F18" s="126"/>
-      <c r="G18" s="126"/>
-      <c r="H18" s="127"/>
+      <c r="C18" s="125"/>
+      <c r="D18" s="125"/>
+      <c r="E18" s="125"/>
+      <c r="F18" s="125"/>
+      <c r="G18" s="125"/>
+      <c r="H18" s="126"/>
     </row>
     <row r="19" spans="1:8" ht="17" customHeight="1">
       <c r="A19" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="128" t="s">
+      <c r="B19" s="127" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="129"/>
-      <c r="D19" s="129"/>
-      <c r="E19" s="129"/>
-      <c r="F19" s="129"/>
-      <c r="G19" s="129"/>
-      <c r="H19" s="130"/>
+      <c r="C19" s="128"/>
+      <c r="D19" s="128"/>
+      <c r="E19" s="128"/>
+      <c r="F19" s="128"/>
+      <c r="G19" s="128"/>
+      <c r="H19" s="129"/>
     </row>
     <row r="21" spans="1:8" ht="15.5">
-      <c r="A21" s="115" t="s">
+      <c r="A21" s="117" t="s">
         <v>69</v>
       </c>
-      <c r="B21" s="115"/>
-      <c r="C21" s="115"/>
-      <c r="D21" s="115"/>
-      <c r="E21" s="115"/>
-      <c r="F21" s="115"/>
-      <c r="G21" s="115"/>
-      <c r="H21" s="115"/>
+      <c r="B21" s="117"/>
+      <c r="C21" s="117"/>
+      <c r="D21" s="117"/>
+      <c r="E21" s="117"/>
+      <c r="F21" s="117"/>
+      <c r="G21" s="117"/>
+      <c r="H21" s="117"/>
     </row>
     <row r="22" spans="1:8" ht="28">
       <c r="A22" s="1" t="s">
@@ -3586,12 +3583,12 @@
       <c r="D22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="131" t="s">
+      <c r="E22" s="122" t="s">
         <v>71</v>
       </c>
-      <c r="F22" s="131"/>
-      <c r="G22" s="131"/>
-      <c r="H22" s="110"/>
+      <c r="F22" s="122"/>
+      <c r="G22" s="122"/>
+      <c r="H22" s="123"/>
     </row>
     <row r="23" spans="1:8" ht="23" customHeight="1">
       <c r="A23" s="10" t="s">
@@ -3606,12 +3603,12 @@
       <c r="D23" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="132" t="s">
+      <c r="E23" s="120" t="s">
         <v>73</v>
       </c>
-      <c r="F23" s="132"/>
-      <c r="G23" s="132"/>
-      <c r="H23" s="133"/>
+      <c r="F23" s="120"/>
+      <c r="G23" s="120"/>
+      <c r="H23" s="121"/>
     </row>
     <row r="24" spans="1:8" ht="23" customHeight="1">
       <c r="A24" s="4" t="s">
@@ -3626,12 +3623,12 @@
       <c r="D24" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="134" t="s">
+      <c r="E24" s="118" t="s">
         <v>75</v>
       </c>
-      <c r="F24" s="134"/>
-      <c r="G24" s="134"/>
-      <c r="H24" s="135"/>
+      <c r="F24" s="118"/>
+      <c r="G24" s="118"/>
+      <c r="H24" s="119"/>
     </row>
     <row r="25" spans="1:8" ht="23" customHeight="1">
       <c r="A25" s="10" t="s">
@@ -3646,12 +3643,12 @@
       <c r="D25" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="132" t="s">
+      <c r="E25" s="120" t="s">
         <v>77</v>
       </c>
-      <c r="F25" s="132"/>
-      <c r="G25" s="132"/>
-      <c r="H25" s="133"/>
+      <c r="F25" s="120"/>
+      <c r="G25" s="120"/>
+      <c r="H25" s="121"/>
     </row>
     <row r="26" spans="1:8" ht="40.5" customHeight="1">
       <c r="A26" s="4" t="s">
@@ -3666,24 +3663,24 @@
       <c r="D26" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="134" t="s">
+      <c r="E26" s="118" t="s">
         <v>79</v>
       </c>
-      <c r="F26" s="134"/>
-      <c r="G26" s="134"/>
-      <c r="H26" s="135"/>
+      <c r="F26" s="118"/>
+      <c r="G26" s="118"/>
+      <c r="H26" s="119"/>
     </row>
     <row r="28" spans="1:8" ht="15.5">
-      <c r="A28" s="115" t="s">
+      <c r="A28" s="117" t="s">
         <v>80</v>
       </c>
-      <c r="B28" s="115"/>
-      <c r="C28" s="115"/>
-      <c r="D28" s="115"/>
-      <c r="E28" s="115"/>
-      <c r="F28" s="115"/>
-      <c r="G28" s="115"/>
-      <c r="H28" s="115"/>
+      <c r="B28" s="117"/>
+      <c r="C28" s="117"/>
+      <c r="D28" s="117"/>
+      <c r="E28" s="117"/>
+      <c r="F28" s="117"/>
+      <c r="G28" s="117"/>
+      <c r="H28" s="117"/>
     </row>
     <row r="29" spans="1:8" ht="28">
       <c r="A29" s="1" t="s">
@@ -3701,9 +3698,9 @@
       <c r="E29" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="F29" s="131"/>
-      <c r="G29" s="131"/>
-      <c r="H29" s="110"/>
+      <c r="F29" s="122"/>
+      <c r="G29" s="122"/>
+      <c r="H29" s="123"/>
     </row>
     <row r="30" spans="1:8" ht="53.5" customHeight="1">
       <c r="A30" s="40" t="s">
@@ -3721,9 +3718,9 @@
       <c r="E30" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="F30" s="132"/>
-      <c r="G30" s="132"/>
-      <c r="H30" s="133"/>
+      <c r="F30" s="120"/>
+      <c r="G30" s="120"/>
+      <c r="H30" s="121"/>
     </row>
     <row r="31" spans="1:8" ht="32" customHeight="1">
       <c r="A31" s="41" t="s">
@@ -3741,9 +3738,9 @@
       <c r="E31" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="F31" s="134"/>
-      <c r="G31" s="134"/>
-      <c r="H31" s="135"/>
+      <c r="F31" s="118"/>
+      <c r="G31" s="118"/>
+      <c r="H31" s="119"/>
     </row>
     <row r="32" spans="1:8" ht="32" customHeight="1">
       <c r="A32" s="40" t="s">
@@ -3761,9 +3758,9 @@
       <c r="E32" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="F32" s="132"/>
-      <c r="G32" s="132"/>
-      <c r="H32" s="133"/>
+      <c r="F32" s="120"/>
+      <c r="G32" s="120"/>
+      <c r="H32" s="121"/>
     </row>
     <row r="33" spans="1:8" ht="32" customHeight="1">
       <c r="A33" s="41" t="s">
@@ -3781,9 +3778,9 @@
       <c r="E33" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="F33" s="134"/>
-      <c r="G33" s="134"/>
-      <c r="H33" s="135"/>
+      <c r="F33" s="118"/>
+      <c r="G33" s="118"/>
+      <c r="H33" s="119"/>
     </row>
     <row r="34" spans="1:8" ht="32" customHeight="1">
       <c r="A34" s="40" t="s">
@@ -3801,9 +3798,9 @@
       <c r="E34" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="F34" s="132"/>
-      <c r="G34" s="132"/>
-      <c r="H34" s="133"/>
+      <c r="F34" s="120"/>
+      <c r="G34" s="120"/>
+      <c r="H34" s="121"/>
     </row>
     <row r="35" spans="1:8" ht="32" customHeight="1">
       <c r="A35" s="41" t="s">
@@ -3821,9 +3818,9 @@
       <c r="E35" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F35" s="134"/>
-      <c r="G35" s="134"/>
-      <c r="H35" s="135"/>
+      <c r="F35" s="118"/>
+      <c r="G35" s="118"/>
+      <c r="H35" s="119"/>
     </row>
     <row r="36" spans="1:8" ht="32" customHeight="1">
       <c r="A36" s="40" t="s">
@@ -3841,138 +3838,110 @@
       <c r="E36" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="F36" s="132"/>
-      <c r="G36" s="132"/>
-      <c r="H36" s="133"/>
+      <c r="F36" s="120"/>
+      <c r="G36" s="120"/>
+      <c r="H36" s="121"/>
     </row>
     <row r="38" spans="1:8" ht="15.5">
-      <c r="A38" s="115" t="s">
+      <c r="A38" s="117" t="s">
         <v>98</v>
       </c>
-      <c r="B38" s="115"/>
-      <c r="C38" s="115"/>
-      <c r="D38" s="115"/>
-      <c r="E38" s="115"/>
-      <c r="F38" s="115"/>
-      <c r="G38" s="115"/>
-      <c r="H38" s="115"/>
+      <c r="B38" s="117"/>
+      <c r="C38" s="117"/>
+      <c r="D38" s="117"/>
+      <c r="E38" s="117"/>
+      <c r="F38" s="117"/>
+      <c r="G38" s="117"/>
+      <c r="H38" s="117"/>
     </row>
     <row r="39" spans="1:8">
-      <c r="A39" s="136" t="s">
+      <c r="A39" s="108" t="s">
         <v>99</v>
       </c>
-      <c r="B39" s="137"/>
-      <c r="C39" s="137"/>
-      <c r="D39" s="137"/>
-      <c r="E39" s="137"/>
-      <c r="F39" s="137"/>
-      <c r="G39" s="137"/>
-      <c r="H39" s="138"/>
+      <c r="B39" s="109"/>
+      <c r="C39" s="109"/>
+      <c r="D39" s="109"/>
+      <c r="E39" s="109"/>
+      <c r="F39" s="109"/>
+      <c r="G39" s="109"/>
+      <c r="H39" s="110"/>
     </row>
     <row r="40" spans="1:8">
-      <c r="A40" s="139"/>
-      <c r="B40" s="140"/>
-      <c r="C40" s="140"/>
-      <c r="D40" s="140"/>
-      <c r="E40" s="140"/>
-      <c r="F40" s="140"/>
-      <c r="G40" s="140"/>
-      <c r="H40" s="141"/>
+      <c r="A40" s="111"/>
+      <c r="B40" s="112"/>
+      <c r="C40" s="112"/>
+      <c r="D40" s="112"/>
+      <c r="E40" s="112"/>
+      <c r="F40" s="112"/>
+      <c r="G40" s="112"/>
+      <c r="H40" s="113"/>
     </row>
     <row r="41" spans="1:8">
-      <c r="A41" s="139"/>
-      <c r="B41" s="140"/>
-      <c r="C41" s="140"/>
-      <c r="D41" s="140"/>
-      <c r="E41" s="140"/>
-      <c r="F41" s="140"/>
-      <c r="G41" s="140"/>
-      <c r="H41" s="141"/>
+      <c r="A41" s="111"/>
+      <c r="B41" s="112"/>
+      <c r="C41" s="112"/>
+      <c r="D41" s="112"/>
+      <c r="E41" s="112"/>
+      <c r="F41" s="112"/>
+      <c r="G41" s="112"/>
+      <c r="H41" s="113"/>
     </row>
     <row r="42" spans="1:8">
-      <c r="A42" s="142"/>
-      <c r="B42" s="143"/>
-      <c r="C42" s="143"/>
-      <c r="D42" s="143"/>
-      <c r="E42" s="143"/>
-      <c r="F42" s="143"/>
-      <c r="G42" s="143"/>
-      <c r="H42" s="144"/>
+      <c r="A42" s="114"/>
+      <c r="B42" s="115"/>
+      <c r="C42" s="115"/>
+      <c r="D42" s="115"/>
+      <c r="E42" s="115"/>
+      <c r="F42" s="115"/>
+      <c r="G42" s="115"/>
+      <c r="H42" s="116"/>
     </row>
     <row r="44" spans="1:8" ht="15.5">
-      <c r="A44" s="115" t="s">
+      <c r="A44" s="117" t="s">
         <v>100</v>
       </c>
-      <c r="B44" s="115"/>
-      <c r="C44" s="115"/>
-      <c r="D44" s="115"/>
-      <c r="E44" s="115"/>
-      <c r="F44" s="115"/>
-      <c r="G44" s="115"/>
-      <c r="H44" s="115"/>
+      <c r="B44" s="117"/>
+      <c r="C44" s="117"/>
+      <c r="D44" s="117"/>
+      <c r="E44" s="117"/>
+      <c r="F44" s="117"/>
+      <c r="G44" s="117"/>
+      <c r="H44" s="117"/>
     </row>
     <row r="45" spans="1:8">
-      <c r="A45" s="136" t="s">
+      <c r="A45" s="108" t="s">
         <v>101</v>
       </c>
-      <c r="B45" s="137"/>
-      <c r="C45" s="137"/>
-      <c r="D45" s="137"/>
-      <c r="E45" s="137"/>
-      <c r="F45" s="137"/>
-      <c r="G45" s="137"/>
-      <c r="H45" s="138"/>
+      <c r="B45" s="109"/>
+      <c r="C45" s="109"/>
+      <c r="D45" s="109"/>
+      <c r="E45" s="109"/>
+      <c r="F45" s="109"/>
+      <c r="G45" s="109"/>
+      <c r="H45" s="110"/>
     </row>
     <row r="46" spans="1:8">
-      <c r="A46" s="139"/>
-      <c r="B46" s="140"/>
-      <c r="C46" s="140"/>
-      <c r="D46" s="140"/>
-      <c r="E46" s="140"/>
-      <c r="F46" s="140"/>
-      <c r="G46" s="140"/>
-      <c r="H46" s="141"/>
+      <c r="A46" s="111"/>
+      <c r="B46" s="112"/>
+      <c r="C46" s="112"/>
+      <c r="D46" s="112"/>
+      <c r="E46" s="112"/>
+      <c r="F46" s="112"/>
+      <c r="G46" s="112"/>
+      <c r="H46" s="113"/>
     </row>
     <row r="47" spans="1:8">
-      <c r="A47" s="142"/>
-      <c r="B47" s="143"/>
-      <c r="C47" s="143"/>
-      <c r="D47" s="143"/>
-      <c r="E47" s="143"/>
-      <c r="F47" s="143"/>
-      <c r="G47" s="143"/>
-      <c r="H47" s="144"/>
+      <c r="A47" s="114"/>
+      <c r="B47" s="115"/>
+      <c r="C47" s="115"/>
+      <c r="D47" s="115"/>
+      <c r="E47" s="115"/>
+      <c r="F47" s="115"/>
+      <c r="G47" s="115"/>
+      <c r="H47" s="116"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="A39:H42"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A45:H47"/>
-    <mergeCell ref="F33:H33"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="F31:H31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="E22:H22"/>
-    <mergeCell ref="E23:H23"/>
-    <mergeCell ref="E24:H24"/>
-    <mergeCell ref="E25:H25"/>
-    <mergeCell ref="E26:H26"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A9:H11"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B15:H15"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:B4"/>
@@ -3983,6 +3952,34 @@
     <mergeCell ref="E5:F6"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="G5:H6"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A9:H11"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="E22:H22"/>
+    <mergeCell ref="E23:H23"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="E25:H25"/>
+    <mergeCell ref="E26:H26"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="A39:H42"/>
+    <mergeCell ref="A44:H44"/>
+    <mergeCell ref="A45:H47"/>
+    <mergeCell ref="F33:H33"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="A38:H38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4003,26 +4000,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17" customHeight="1">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="139" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
     </row>
     <row r="3" spans="1:7" ht="15.5">
-      <c r="A3" s="115" t="s">
+      <c r="A3" s="117" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="115"/>
-      <c r="C3" s="115"/>
-      <c r="D3" s="115"/>
-      <c r="E3" s="115"/>
-      <c r="F3" s="115"/>
-      <c r="G3" s="115"/>
+      <c r="B3" s="117"/>
+      <c r="C3" s="117"/>
+      <c r="D3" s="117"/>
+      <c r="E3" s="117"/>
+      <c r="F3" s="117"/>
+      <c r="G3" s="117"/>
     </row>
     <row r="4" spans="1:7" ht="28">
       <c r="A4" s="1" t="s">
@@ -4034,12 +4031,12 @@
       <c r="C4" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D4" s="131" t="s">
+      <c r="D4" s="122" t="s">
         <v>107</v>
       </c>
-      <c r="E4" s="131"/>
-      <c r="F4" s="131"/>
-      <c r="G4" s="110"/>
+      <c r="E4" s="122"/>
+      <c r="F4" s="122"/>
+      <c r="G4" s="123"/>
     </row>
     <row r="5" spans="1:7" ht="32" customHeight="1">
       <c r="A5" s="10" t="s">
@@ -4051,12 +4048,12 @@
       <c r="C5" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D5" s="132" t="s">
+      <c r="D5" s="120" t="s">
         <v>111</v>
       </c>
-      <c r="E5" s="132"/>
-      <c r="F5" s="132"/>
-      <c r="G5" s="133"/>
+      <c r="E5" s="120"/>
+      <c r="F5" s="120"/>
+      <c r="G5" s="121"/>
     </row>
     <row r="6" spans="1:7" ht="48" customHeight="1">
       <c r="A6" s="4" t="s">
@@ -4068,12 +4065,12 @@
       <c r="C6" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D6" s="134" t="s">
+      <c r="D6" s="118" t="s">
         <v>114</v>
       </c>
-      <c r="E6" s="134"/>
-      <c r="F6" s="134"/>
-      <c r="G6" s="135"/>
+      <c r="E6" s="118"/>
+      <c r="F6" s="118"/>
+      <c r="G6" s="119"/>
     </row>
     <row r="7" spans="1:7" ht="42.5" customHeight="1">
       <c r="A7" s="10" t="s">
@@ -4085,16 +4082,16 @@
       <c r="C7" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D7" s="132" t="s">
+      <c r="D7" s="120" t="s">
         <v>117</v>
       </c>
-      <c r="E7" s="132"/>
-      <c r="F7" s="132"/>
-      <c r="G7" s="133"/>
+      <c r="E7" s="120"/>
+      <c r="F7" s="120"/>
+      <c r="G7" s="121"/>
     </row>
     <row r="8" spans="1:7" ht="52" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>118</v>
@@ -4102,23 +4099,23 @@
       <c r="C8" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D8" s="134" t="s">
+      <c r="D8" s="118" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="134"/>
-      <c r="F8" s="134"/>
-      <c r="G8" s="135"/>
+      <c r="E8" s="118"/>
+      <c r="F8" s="118"/>
+      <c r="G8" s="119"/>
     </row>
     <row r="10" spans="1:7" ht="15.5">
-      <c r="A10" s="115" t="s">
+      <c r="A10" s="117" t="s">
         <v>120</v>
       </c>
-      <c r="B10" s="115"/>
-      <c r="C10" s="115"/>
-      <c r="D10" s="115"/>
-      <c r="E10" s="115"/>
-      <c r="F10" s="115"/>
-      <c r="G10" s="115"/>
+      <c r="B10" s="117"/>
+      <c r="C10" s="117"/>
+      <c r="D10" s="117"/>
+      <c r="E10" s="117"/>
+      <c r="F10" s="117"/>
+      <c r="G10" s="117"/>
     </row>
     <row r="11" spans="1:7" ht="25.5" customHeight="1">
       <c r="A11" s="1" t="s">
@@ -4130,46 +4127,46 @@
       <c r="C11" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D11" s="131" t="s">
-        <v>326</v>
-      </c>
-      <c r="E11" s="131"/>
-      <c r="F11" s="131"/>
-      <c r="G11" s="110"/>
+      <c r="D11" s="122" t="s">
+        <v>325</v>
+      </c>
+      <c r="E11" s="122"/>
+      <c r="F11" s="122"/>
+      <c r="G11" s="123"/>
     </row>
     <row r="12" spans="1:7" ht="46" customHeight="1">
       <c r="A12" s="66" t="s">
         <v>124</v>
       </c>
       <c r="B12" s="67" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C12" s="66" t="s">
-        <v>325</v>
-      </c>
-      <c r="D12" s="145" t="s">
         <v>324</v>
       </c>
-      <c r="E12" s="145"/>
-      <c r="F12" s="145"/>
-      <c r="G12" s="146"/>
+      <c r="D12" s="146" t="s">
+        <v>323</v>
+      </c>
+      <c r="E12" s="146"/>
+      <c r="F12" s="146"/>
+      <c r="G12" s="147"/>
     </row>
     <row r="13" spans="1:7" ht="58" customHeight="1">
       <c r="A13" s="66" t="s">
         <v>124</v>
       </c>
       <c r="B13" s="67" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C13" s="66" t="s">
-        <v>322</v>
-      </c>
-      <c r="D13" s="145" t="s">
-        <v>338</v>
-      </c>
-      <c r="E13" s="145"/>
-      <c r="F13" s="145"/>
-      <c r="G13" s="146"/>
+        <v>321</v>
+      </c>
+      <c r="D13" s="146" t="s">
+        <v>337</v>
+      </c>
+      <c r="E13" s="146"/>
+      <c r="F13" s="146"/>
+      <c r="G13" s="147"/>
     </row>
     <row r="14" spans="1:7" ht="31" customHeight="1">
       <c r="A14" s="66" t="s">
@@ -4179,48 +4176,48 @@
         <v>112</v>
       </c>
       <c r="C14" s="66" t="s">
-        <v>325</v>
-      </c>
-      <c r="D14" s="145" t="s">
         <v>324</v>
       </c>
-      <c r="E14" s="145"/>
-      <c r="F14" s="145"/>
-      <c r="G14" s="146"/>
+      <c r="D14" s="146" t="s">
+        <v>323</v>
+      </c>
+      <c r="E14" s="146"/>
+      <c r="F14" s="146"/>
+      <c r="G14" s="147"/>
     </row>
     <row r="15" spans="1:7" ht="43" customHeight="1">
       <c r="A15" s="66" t="s">
         <v>124</v>
       </c>
       <c r="B15" s="67" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C15" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="145" t="s">
-        <v>340</v>
-      </c>
-      <c r="E15" s="145"/>
-      <c r="F15" s="145"/>
-      <c r="G15" s="146"/>
+      <c r="D15" s="146" t="s">
+        <v>339</v>
+      </c>
+      <c r="E15" s="146"/>
+      <c r="F15" s="146"/>
+      <c r="G15" s="147"/>
     </row>
     <row r="16" spans="1:7" ht="33" customHeight="1">
       <c r="A16" s="66" t="s">
         <v>124</v>
       </c>
       <c r="B16" s="68" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C16" s="66" t="s">
-        <v>323</v>
-      </c>
-      <c r="D16" s="145" t="s">
-        <v>334</v>
-      </c>
-      <c r="E16" s="145"/>
-      <c r="F16" s="145"/>
-      <c r="G16" s="146"/>
+        <v>322</v>
+      </c>
+      <c r="D16" s="146" t="s">
+        <v>333</v>
+      </c>
+      <c r="E16" s="146"/>
+      <c r="F16" s="146"/>
+      <c r="G16" s="147"/>
     </row>
     <row r="17" spans="1:7" ht="33.5" customHeight="1">
       <c r="A17" s="69" t="s">
@@ -4232,12 +4229,12 @@
       <c r="C17" s="66" t="s">
         <v>127</v>
       </c>
-      <c r="D17" s="145" t="s">
-        <v>335</v>
-      </c>
-      <c r="E17" s="145"/>
-      <c r="F17" s="145"/>
-      <c r="G17" s="146"/>
+      <c r="D17" s="146" t="s">
+        <v>334</v>
+      </c>
+      <c r="E17" s="146"/>
+      <c r="F17" s="146"/>
+      <c r="G17" s="147"/>
     </row>
     <row r="18" spans="1:7" ht="32" customHeight="1">
       <c r="A18" s="69" t="s">
@@ -4249,12 +4246,12 @@
       <c r="C18" s="66" t="s">
         <v>130</v>
       </c>
-      <c r="D18" s="145" t="s">
-        <v>336</v>
-      </c>
-      <c r="E18" s="145"/>
-      <c r="F18" s="145"/>
-      <c r="G18" s="146"/>
+      <c r="D18" s="146" t="s">
+        <v>335</v>
+      </c>
+      <c r="E18" s="146"/>
+      <c r="F18" s="146"/>
+      <c r="G18" s="147"/>
     </row>
     <row r="19" spans="1:7" ht="30.5" customHeight="1">
       <c r="A19" s="69" t="s">
@@ -4266,12 +4263,12 @@
       <c r="C19" s="66" t="s">
         <v>132</v>
       </c>
-      <c r="D19" s="145" t="s">
-        <v>339</v>
-      </c>
-      <c r="E19" s="145"/>
-      <c r="F19" s="145"/>
-      <c r="G19" s="146"/>
+      <c r="D19" s="146" t="s">
+        <v>338</v>
+      </c>
+      <c r="E19" s="146"/>
+      <c r="F19" s="146"/>
+      <c r="G19" s="147"/>
     </row>
     <row r="20" spans="1:7" ht="44" customHeight="1">
       <c r="A20" s="69" t="s">
@@ -4283,23 +4280,23 @@
       <c r="C20" s="66" t="s">
         <v>134</v>
       </c>
-      <c r="D20" s="145" t="s">
-        <v>337</v>
-      </c>
-      <c r="E20" s="145"/>
-      <c r="F20" s="145"/>
-      <c r="G20" s="146"/>
+      <c r="D20" s="146" t="s">
+        <v>336</v>
+      </c>
+      <c r="E20" s="146"/>
+      <c r="F20" s="146"/>
+      <c r="G20" s="147"/>
     </row>
     <row r="23" spans="1:7" ht="15.5">
-      <c r="A23" s="115" t="s">
+      <c r="A23" s="117" t="s">
         <v>135</v>
       </c>
-      <c r="B23" s="115"/>
-      <c r="C23" s="115"/>
-      <c r="D23" s="115"/>
-      <c r="E23" s="115"/>
-      <c r="F23" s="115"/>
-      <c r="G23" s="115"/>
+      <c r="B23" s="117"/>
+      <c r="C23" s="117"/>
+      <c r="D23" s="117"/>
+      <c r="E23" s="117"/>
+      <c r="F23" s="117"/>
+      <c r="G23" s="117"/>
     </row>
     <row r="24" spans="1:7" ht="42">
       <c r="A24" s="1" t="s">
@@ -4314,11 +4311,11 @@
       <c r="D24" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E24" s="131" t="s">
+      <c r="E24" s="122" t="s">
         <v>138</v>
       </c>
-      <c r="F24" s="131"/>
-      <c r="G24" s="110"/>
+      <c r="F24" s="122"/>
+      <c r="G24" s="123"/>
     </row>
     <row r="25" spans="1:7" ht="24" customHeight="1">
       <c r="A25" s="40" t="s">
@@ -4333,11 +4330,11 @@
       <c r="D25" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="132" t="s">
+      <c r="E25" s="120" t="s">
         <v>142</v>
       </c>
-      <c r="F25" s="132"/>
-      <c r="G25" s="133"/>
+      <c r="F25" s="120"/>
+      <c r="G25" s="121"/>
     </row>
     <row r="26" spans="1:7" ht="24" customHeight="1">
       <c r="A26" s="41" t="s">
@@ -4352,11 +4349,11 @@
       <c r="D26" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="134" t="s">
+      <c r="E26" s="118" t="s">
         <v>146</v>
       </c>
-      <c r="F26" s="134"/>
-      <c r="G26" s="135"/>
+      <c r="F26" s="118"/>
+      <c r="G26" s="119"/>
     </row>
     <row r="27" spans="1:7" ht="24" customHeight="1">
       <c r="A27" s="40" t="s">
@@ -4371,11 +4368,11 @@
       <c r="D27" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="132" t="s">
+      <c r="E27" s="120" t="s">
         <v>149</v>
       </c>
-      <c r="F27" s="132"/>
-      <c r="G27" s="133"/>
+      <c r="F27" s="120"/>
+      <c r="G27" s="121"/>
     </row>
     <row r="28" spans="1:7" ht="24" customHeight="1">
       <c r="A28" s="41" t="s">
@@ -4390,11 +4387,11 @@
       <c r="D28" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E28" s="134" t="s">
+      <c r="E28" s="118" t="s">
         <v>151</v>
       </c>
-      <c r="F28" s="134"/>
-      <c r="G28" s="135"/>
+      <c r="F28" s="118"/>
+      <c r="G28" s="119"/>
     </row>
     <row r="29" spans="1:7" ht="24" customHeight="1">
       <c r="A29" s="40" t="s">
@@ -4409,11 +4406,11 @@
       <c r="D29" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="132" t="s">
+      <c r="E29" s="120" t="s">
         <v>155</v>
       </c>
-      <c r="F29" s="132"/>
-      <c r="G29" s="133"/>
+      <c r="F29" s="120"/>
+      <c r="G29" s="121"/>
     </row>
     <row r="30" spans="1:7" ht="24" customHeight="1">
       <c r="A30" s="41" t="s">
@@ -4428,11 +4425,11 @@
       <c r="D30" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="134" t="s">
+      <c r="E30" s="118" t="s">
         <v>158</v>
       </c>
-      <c r="F30" s="134"/>
-      <c r="G30" s="135"/>
+      <c r="F30" s="118"/>
+      <c r="G30" s="119"/>
     </row>
     <row r="31" spans="1:7" ht="24" customHeight="1">
       <c r="A31" s="40" t="s">
@@ -4447,24 +4444,19 @@
       <c r="D31" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="132" t="s">
+      <c r="E31" s="120" t="s">
         <v>161</v>
       </c>
-      <c r="F31" s="132"/>
-      <c r="G31" s="133"/>
+      <c r="F31" s="120"/>
+      <c r="G31" s="121"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="A23:G23"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="D6:G6"/>
     <mergeCell ref="D13:G13"/>
     <mergeCell ref="D17:G17"/>
     <mergeCell ref="D18:G18"/>
@@ -4477,11 +4469,16 @@
     <mergeCell ref="D14:G14"/>
     <mergeCell ref="D15:G15"/>
     <mergeCell ref="D16:G16"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="D4:G4"/>
-    <mergeCell ref="D5:G5"/>
-    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="E31:G31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4500,28 +4497,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17" customHeight="1">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="139" t="s">
         <v>162</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
     </row>
     <row r="3" spans="1:8" ht="22" customHeight="1">
-      <c r="A3" s="147" t="s">
+      <c r="A3" s="157" t="s">
         <v>163</v>
       </c>
-      <c r="B3" s="148"/>
-      <c r="C3" s="148"/>
-      <c r="D3" s="148"/>
-      <c r="E3" s="148"/>
-      <c r="F3" s="148"/>
-      <c r="G3" s="148"/>
-      <c r="H3" s="149"/>
+      <c r="B3" s="158"/>
+      <c r="C3" s="158"/>
+      <c r="D3" s="158"/>
+      <c r="E3" s="158"/>
+      <c r="F3" s="158"/>
+      <c r="G3" s="158"/>
+      <c r="H3" s="159"/>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
@@ -4539,11 +4536,11 @@
       <c r="E5" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="F5" s="131" t="s">
+      <c r="F5" s="122" t="s">
         <v>169</v>
       </c>
-      <c r="G5" s="131"/>
-      <c r="H5" s="110"/>
+      <c r="G5" s="122"/>
+      <c r="H5" s="123"/>
     </row>
     <row r="6" spans="1:8" ht="33" customHeight="1">
       <c r="A6" s="10" t="s">
@@ -4561,11 +4558,11 @@
       <c r="E6" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="F6" s="132" t="s">
+      <c r="F6" s="120" t="s">
         <v>174</v>
       </c>
-      <c r="G6" s="132"/>
-      <c r="H6" s="133"/>
+      <c r="G6" s="120"/>
+      <c r="H6" s="121"/>
     </row>
     <row r="7" spans="1:8" ht="33" customHeight="1">
       <c r="A7" s="4" t="s">
@@ -4583,11 +4580,11 @@
       <c r="E7" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="F7" s="134" t="s">
+      <c r="F7" s="118" t="s">
         <v>178</v>
       </c>
-      <c r="G7" s="134"/>
-      <c r="H7" s="135"/>
+      <c r="G7" s="118"/>
+      <c r="H7" s="119"/>
     </row>
     <row r="8" spans="1:8" ht="33" customHeight="1">
       <c r="A8" s="10" t="s">
@@ -4605,11 +4602,11 @@
       <c r="E8" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="F8" s="132" t="s">
+      <c r="F8" s="120" t="s">
         <v>183</v>
       </c>
-      <c r="G8" s="132"/>
-      <c r="H8" s="133"/>
+      <c r="G8" s="120"/>
+      <c r="H8" s="121"/>
     </row>
     <row r="9" spans="1:8" ht="33" customHeight="1">
       <c r="A9" s="4" t="s">
@@ -4627,11 +4624,11 @@
       <c r="E9" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="F9" s="134" t="s">
+      <c r="F9" s="118" t="s">
         <v>187</v>
       </c>
-      <c r="G9" s="134"/>
-      <c r="H9" s="135"/>
+      <c r="G9" s="118"/>
+      <c r="H9" s="119"/>
     </row>
     <row r="10" spans="1:8" ht="33" customHeight="1">
       <c r="A10" s="10" t="s">
@@ -4649,11 +4646,11 @@
       <c r="E10" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="F10" s="132" t="s">
+      <c r="F10" s="120" t="s">
         <v>192</v>
       </c>
-      <c r="G10" s="132"/>
-      <c r="H10" s="133"/>
+      <c r="G10" s="120"/>
+      <c r="H10" s="121"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="42" t="s">
@@ -4671,60 +4668,60 @@
       <c r="H11" s="44"/>
     </row>
     <row r="13" spans="1:8" ht="15.5">
-      <c r="A13" s="115" t="s">
+      <c r="A13" s="117" t="s">
         <v>194</v>
       </c>
-      <c r="B13" s="115"/>
-      <c r="C13" s="115"/>
-      <c r="D13" s="115"/>
-      <c r="E13" s="115"/>
-      <c r="F13" s="115"/>
-      <c r="G13" s="115"/>
-      <c r="H13" s="115"/>
+      <c r="B13" s="117"/>
+      <c r="C13" s="117"/>
+      <c r="D13" s="117"/>
+      <c r="E13" s="117"/>
+      <c r="F13" s="117"/>
+      <c r="G13" s="117"/>
+      <c r="H13" s="117"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="136" t="s">
+      <c r="A14" s="108" t="s">
         <v>195</v>
       </c>
-      <c r="B14" s="137"/>
-      <c r="C14" s="137"/>
-      <c r="D14" s="137"/>
-      <c r="E14" s="137"/>
-      <c r="F14" s="137"/>
-      <c r="G14" s="137"/>
-      <c r="H14" s="138"/>
+      <c r="B14" s="109"/>
+      <c r="C14" s="109"/>
+      <c r="D14" s="109"/>
+      <c r="E14" s="109"/>
+      <c r="F14" s="109"/>
+      <c r="G14" s="109"/>
+      <c r="H14" s="110"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="139"/>
-      <c r="B15" s="140"/>
-      <c r="C15" s="140"/>
-      <c r="D15" s="140"/>
-      <c r="E15" s="140"/>
-      <c r="F15" s="140"/>
-      <c r="G15" s="140"/>
-      <c r="H15" s="141"/>
+      <c r="A15" s="111"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
+      <c r="G15" s="112"/>
+      <c r="H15" s="113"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="142"/>
-      <c r="B16" s="143"/>
-      <c r="C16" s="143"/>
-      <c r="D16" s="143"/>
-      <c r="E16" s="143"/>
-      <c r="F16" s="143"/>
-      <c r="G16" s="143"/>
-      <c r="H16" s="144"/>
+      <c r="A16" s="114"/>
+      <c r="B16" s="115"/>
+      <c r="C16" s="115"/>
+      <c r="D16" s="115"/>
+      <c r="E16" s="115"/>
+      <c r="F16" s="115"/>
+      <c r="G16" s="115"/>
+      <c r="H16" s="116"/>
     </row>
     <row r="18" spans="1:8" ht="15.5">
-      <c r="A18" s="115" t="s">
+      <c r="A18" s="117" t="s">
         <v>196</v>
       </c>
-      <c r="B18" s="115"/>
-      <c r="C18" s="115"/>
-      <c r="D18" s="115"/>
-      <c r="E18" s="115"/>
-      <c r="F18" s="115"/>
-      <c r="G18" s="115"/>
-      <c r="H18" s="115"/>
+      <c r="B18" s="117"/>
+      <c r="C18" s="117"/>
+      <c r="D18" s="117"/>
+      <c r="E18" s="117"/>
+      <c r="F18" s="117"/>
+      <c r="G18" s="117"/>
+      <c r="H18" s="117"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="1" t="s">
@@ -4797,61 +4794,66 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="15.5">
-      <c r="A25" s="115" t="s">
+      <c r="A25" s="117" t="s">
         <v>217</v>
       </c>
-      <c r="B25" s="115"/>
-      <c r="C25" s="115"/>
-      <c r="D25" s="115"/>
-      <c r="E25" s="115"/>
-      <c r="F25" s="115"/>
-      <c r="G25" s="115"/>
-      <c r="H25" s="115"/>
+      <c r="B25" s="117"/>
+      <c r="C25" s="117"/>
+      <c r="D25" s="117"/>
+      <c r="E25" s="117"/>
+      <c r="F25" s="117"/>
+      <c r="G25" s="117"/>
+      <c r="H25" s="117"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="150" t="s">
+      <c r="A26" s="148" t="s">
         <v>218</v>
       </c>
-      <c r="B26" s="151"/>
-      <c r="C26" s="151"/>
-      <c r="D26" s="151"/>
-      <c r="E26" s="151"/>
-      <c r="F26" s="151"/>
-      <c r="G26" s="151"/>
-      <c r="H26" s="152"/>
+      <c r="B26" s="149"/>
+      <c r="C26" s="149"/>
+      <c r="D26" s="149"/>
+      <c r="E26" s="149"/>
+      <c r="F26" s="149"/>
+      <c r="G26" s="149"/>
+      <c r="H26" s="150"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="153"/>
-      <c r="B27" s="154"/>
-      <c r="C27" s="154"/>
-      <c r="D27" s="154"/>
-      <c r="E27" s="154"/>
-      <c r="F27" s="154"/>
-      <c r="G27" s="154"/>
-      <c r="H27" s="155"/>
+      <c r="A27" s="151"/>
+      <c r="B27" s="152"/>
+      <c r="C27" s="152"/>
+      <c r="D27" s="152"/>
+      <c r="E27" s="152"/>
+      <c r="F27" s="152"/>
+      <c r="G27" s="152"/>
+      <c r="H27" s="153"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="153"/>
-      <c r="B28" s="154"/>
-      <c r="C28" s="154"/>
-      <c r="D28" s="154"/>
-      <c r="E28" s="154"/>
-      <c r="F28" s="154"/>
-      <c r="G28" s="154"/>
-      <c r="H28" s="155"/>
+      <c r="A28" s="151"/>
+      <c r="B28" s="152"/>
+      <c r="C28" s="152"/>
+      <c r="D28" s="152"/>
+      <c r="E28" s="152"/>
+      <c r="F28" s="152"/>
+      <c r="G28" s="152"/>
+      <c r="H28" s="153"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="156"/>
-      <c r="B29" s="157"/>
-      <c r="C29" s="157"/>
-      <c r="D29" s="157"/>
-      <c r="E29" s="157"/>
-      <c r="F29" s="157"/>
-      <c r="G29" s="157"/>
-      <c r="H29" s="158"/>
+      <c r="A29" s="154"/>
+      <c r="B29" s="155"/>
+      <c r="C29" s="155"/>
+      <c r="D29" s="155"/>
+      <c r="E29" s="155"/>
+      <c r="F29" s="155"/>
+      <c r="G29" s="155"/>
+      <c r="H29" s="156"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="F7:H7"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A26:H29"/>
@@ -4860,11 +4862,6 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A14:H16"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="F5:H5"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="F7:H7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4885,28 +4882,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17" customHeight="1">
-      <c r="A1" s="107" t="s">
+      <c r="A1" s="139" t="s">
         <v>219</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1">
-      <c r="A2" s="147" t="s">
+      <c r="A2" s="157" t="s">
         <v>220</v>
       </c>
-      <c r="B2" s="148"/>
-      <c r="C2" s="148"/>
-      <c r="D2" s="148"/>
-      <c r="E2" s="148"/>
-      <c r="F2" s="148"/>
-      <c r="G2" s="148"/>
-      <c r="H2" s="149"/>
+      <c r="B2" s="158"/>
+      <c r="C2" s="158"/>
+      <c r="D2" s="158"/>
+      <c r="E2" s="158"/>
+      <c r="F2" s="158"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="159"/>
     </row>
     <row r="4" spans="1:8" ht="22" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -5117,16 +5114,16 @@
       </c>
     </row>
     <row r="14" spans="1:8" ht="15.5">
-      <c r="A14" s="115" t="s">
+      <c r="A14" s="117" t="s">
         <v>262</v>
       </c>
-      <c r="B14" s="115"/>
-      <c r="C14" s="115"/>
-      <c r="D14" s="115"/>
-      <c r="E14" s="115"/>
-      <c r="F14" s="115"/>
-      <c r="G14" s="115"/>
-      <c r="H14" s="115"/>
+      <c r="B14" s="117"/>
+      <c r="C14" s="117"/>
+      <c r="D14" s="117"/>
+      <c r="E14" s="117"/>
+      <c r="F14" s="117"/>
+      <c r="G14" s="117"/>
+      <c r="H14" s="117"/>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="1" t="s">

</xml_diff>